<commit_message>
version en la presentacion 9/7/24
</commit_message>
<xml_diff>
--- a/sistema de registro de docentes/Resources/lista_doc.xlsx
+++ b/sistema de registro de docentes/Resources/lista_doc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROYECTO\proyecto registro de asistencia profesores\sistema de registro de docentes\sistema de registro de docentes\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{307EBDA5-CF3A-49A7-B850-E895E87B6DD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5441E973-6D0A-455D-B566-C0467865372E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5100" yWindow="3012" windowWidth="9600" windowHeight="6348" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja2" sheetId="5" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2838" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2824" uniqueCount="524">
   <si>
     <t>Nº</t>
   </si>
@@ -1576,40 +1576,22 @@
     <t>Estado</t>
   </si>
   <si>
-    <t>ING</t>
-  </si>
-  <si>
-    <t>LEON</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FERNANDO </t>
-  </si>
-  <si>
-    <t>SEXTO SEMESTRE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ROBOTICA </t>
-  </si>
-  <si>
-    <t>OCTAVO SEMESTRE</t>
+    <t>HUANCO</t>
+  </si>
+  <si>
+    <t>QUELCA</t>
+  </si>
+  <si>
+    <t>JULIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANÁLISIS Y DISEÑO DE SISTEMAS BASADOS EN MICROPROCESADORES </t>
+  </si>
+  <si>
+    <t>TERCER SEMESTRE</t>
   </si>
   <si>
     <t>NOVENO SEMESTRE</t>
-  </si>
-  <si>
-    <t>ing</t>
-  </si>
-  <si>
-    <t>colque</t>
-  </si>
-  <si>
-    <t>leon</t>
-  </si>
-  <si>
-    <t>nichar</t>
-  </si>
-  <si>
-    <t>a</t>
   </si>
 </sst>
 </file>
@@ -2277,7 +2259,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U188"/>
+  <dimension ref="A1:U186"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.109375" customWidth="1"/>
@@ -12715,132 +12697,74 @@
         <v>516</v>
       </c>
     </row>
-    <row r="185" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:21" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A185">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="B185" t="s">
+        <v>18</v>
+      </c>
+      <c r="C185" t="s">
         <v>518</v>
       </c>
-      <c r="C185" t="s">
+      <c r="D185" t="s">
         <v>519</v>
-      </c>
-      <c r="D185" t="s">
-        <v>276</v>
       </c>
       <c r="E185" t="s">
         <v>520</v>
       </c>
       <c r="F185">
-        <v>2345644</v>
+        <v>123</v>
       </c>
       <c r="G185" t="s">
-        <v>475</v>
+        <v>387</v>
       </c>
       <c r="H185" t="s">
         <v>521</v>
       </c>
       <c r="I185" t="s">
-        <v>25</v>
-      </c>
-      <c r="P185" t="s">
-        <v>387</v>
+        <v>522</v>
+      </c>
+      <c r="J185" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="U185" t="s">
+        <v>516</v>
       </c>
     </row>
     <row r="186" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A186">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="B186" t="s">
+        <v>18</v>
+      </c>
+      <c r="C186" t="s">
         <v>518</v>
       </c>
-      <c r="C186" t="s">
+      <c r="D186" t="s">
         <v>519</v>
-      </c>
-      <c r="D186" t="s">
-        <v>276</v>
       </c>
       <c r="E186" t="s">
         <v>520</v>
       </c>
       <c r="F186">
-        <v>2345644</v>
+        <v>123</v>
       </c>
       <c r="G186" t="s">
-        <v>522</v>
+        <v>387</v>
       </c>
       <c r="H186" t="s">
+        <v>174</v>
+      </c>
+      <c r="I186" t="s">
         <v>523</v>
       </c>
-      <c r="I186" t="s">
-        <v>25</v>
-      </c>
-      <c r="P186" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="187" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A187">
-        <v>186</v>
-      </c>
-      <c r="B187" t="s">
-        <v>518</v>
-      </c>
-      <c r="C187" t="s">
-        <v>519</v>
-      </c>
-      <c r="D187" t="s">
-        <v>276</v>
-      </c>
-      <c r="E187" t="s">
-        <v>520</v>
-      </c>
-      <c r="F187">
-        <v>2345644</v>
-      </c>
-      <c r="G187" t="s">
-        <v>174</v>
-      </c>
-      <c r="H187" t="s">
-        <v>524</v>
-      </c>
-      <c r="I187" t="s">
-        <v>25</v>
-      </c>
-      <c r="P187" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="188" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A188">
-        <v>187</v>
-      </c>
-      <c r="B188" t="s">
-        <v>525</v>
-      </c>
-      <c r="C188" t="s">
-        <v>526</v>
-      </c>
-      <c r="D188" t="s">
-        <v>527</v>
-      </c>
-      <c r="E188" t="s">
-        <v>528</v>
-      </c>
-      <c r="F188">
-        <v>1231432</v>
-      </c>
-      <c r="G188" t="s">
-        <v>387</v>
-      </c>
-      <c r="H188" t="s">
-        <v>479</v>
-      </c>
-      <c r="I188" t="s">
-        <v>521</v>
-      </c>
-      <c r="J188" s="19" t="s">
-        <v>529</v>
+      <c r="J186" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="U186" t="s">
+        <v>516</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
version 11/7/24 presentacion final
</commit_message>
<xml_diff>
--- a/sistema de registro de docentes/Resources/lista_doc.xlsx
+++ b/sistema de registro de docentes/Resources/lista_doc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROYECTO\proyecto registro de asistencia profesores\sistema de registro de docentes\sistema de registro de docentes\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DE40A67-7957-4DA0-87BE-2C14A4EF2B77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E5E5DC-9751-4BE7-A2E2-AA43D6BA238B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5448" yWindow="3360" windowWidth="9600" windowHeight="6348" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja2" sheetId="5" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2404" uniqueCount="517">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2404" uniqueCount="519">
   <si>
     <t>Nº</t>
   </si>
@@ -1571,6 +1571,12 @@
   </si>
   <si>
     <t>TALLER DE MODELACIÓN Y SIMULACIÓN</t>
+  </si>
+  <si>
+    <t>ING. EN TELECOMUNICACIONES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VARIABLE COMPLEJA </t>
   </si>
 </sst>
 </file>
@@ -2250,13 +2256,13 @@
         <v>24</v>
       </c>
       <c r="F2" s="21">
-        <v>2216676</v>
+        <v>221667600</v>
       </c>
       <c r="G2" s="21" t="s">
-        <v>25</v>
+        <v>517</v>
       </c>
       <c r="H2" s="22" t="s">
-        <v>26</v>
+        <v>518</v>
       </c>
       <c r="I2" s="16" t="s">
         <v>27</v>
@@ -2442,7 +2448,7 @@
       <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
       <c r="U5" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:21" ht="27" customHeight="1" x14ac:dyDescent="0.3">
@@ -2601,7 +2607,7 @@
       <c r="Q8" s="1"/>
       <c r="R8" s="1"/>
       <c r="U8" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:21" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>